<commit_message>
Update ANA/SNIRH app and data snapshot
</commit_message>
<xml_diff>
--- a/0144_Cuenca_Mauri/_raw_reportes_xlsx/IDConfig_64910_completo.xlsx
+++ b/0144_Cuenca_Mauri/_raw_reportes_xlsx/IDConfig_64910_completo.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporte" sheetId="2" r:id="R29e546cfb553460f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporte" sheetId="2" r:id="Rc13844d8840a4bf1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -255,6 +255,141 @@
     <x:row>
       <x:c s="1" t="inlineStr">
         <x:is>
+          <x:t>23/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1233</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>22/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1227</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>21/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1262</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>20/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1289</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>19/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1315</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>18/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1490</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>17/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1301</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>16/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1219</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>15/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1212</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
           <x:t>14/08/2026</x:t>
         </x:is>
       </x:c>

</xml_diff>

<commit_message>
Update monthly ANA-SNIRH snapshot to 2026-10-11
</commit_message>
<xml_diff>
--- a/0144_Cuenca_Mauri/_raw_reportes_xlsx/IDConfig_64910_completo.xlsx
+++ b/0144_Cuenca_Mauri/_raw_reportes_xlsx/IDConfig_64910_completo.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporte" sheetId="2" r:id="Rc13844d8840a4bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporte" sheetId="2" r:id="R03f111e5f0a24d2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -255,6 +255,726 @@
     <x:row>
       <x:c s="1" t="inlineStr">
         <x:is>
+          <x:t>10/10/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.0995</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>09/10/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.0977</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>08/10/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1014</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>07/10/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1386</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>06/10/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1992</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>05/10/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2009</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>04/10/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1967</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>03/10/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1942</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>02/10/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1951</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>01/10/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1992</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>30/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2001</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>29/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>28/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2068</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>27/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2009</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>26/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2018</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>25/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2070</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>24/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2112</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>23/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2068</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>22/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.1975</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>21/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2001</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>20/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2034</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>19/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>18/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2192</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>17/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2068</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>16/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2077</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>15/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2086</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>14/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2068</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>13/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2068</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>12/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2051</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>11/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2043</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>10/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2068</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>09/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2068</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>08/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2068</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>07/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2078</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>06/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2060</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>05/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2077</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>04/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2068</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>03/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2079</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>02/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2098</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>01/09/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2057</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>31/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2063</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>30/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2105</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>29/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2113</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>28/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2105</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>27/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2070</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>26/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2079</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>25/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2149</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
+          <x:t>24/08/2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="7" t="inlineStr">
+        <x:is>
+          <x:t>00:00</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="3">
+        <x:v>      0.2237</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="1" t="inlineStr">
+        <x:is>
           <x:t>23/08/2026</x:t>
         </x:is>
       </x:c>
@@ -264,7 +984,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1233</x:v>
+        <x:v>      0.2148</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -279,7 +999,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1227</x:v>
+        <x:v>      0.2150</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -294,7 +1014,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1262</x:v>
+        <x:v>      0.2169</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -309,7 +1029,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1289</x:v>
+        <x:v>      0.2240</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -324,7 +1044,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1315</x:v>
+        <x:v>      0.2257</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -339,7 +1059,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1490</x:v>
+        <x:v>      0.2484</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -354,7 +1074,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1301</x:v>
+        <x:v>      0.2229</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -369,7 +1089,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1219</x:v>
+        <x:v>      0.2130</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -384,7 +1104,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1212</x:v>
+        <x:v>      0.2121</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -399,7 +1119,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1200</x:v>
+        <x:v>      0.2095</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -414,7 +1134,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1318</x:v>
+        <x:v>      0.2269</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -429,7 +1149,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.1992</x:v>
+        <x:v>      0.2496</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -459,7 +1179,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.2419</x:v>
+        <x:v>      0.2380</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -504,7 +1224,7 @@
         </x:is>
       </x:c>
       <x:c s="3">
-        <x:v>      0.2278</x:v>
+        <x:v>      0.2258</x:v>
       </x:c>
     </x:row>
     <x:row>

</xml_diff>